<commit_message>
Populate workbook with live market data (Stage 4)
</commit_message>
<xml_diff>
--- a/models/builds/2026-08-08-Kaetsu-eur-receivable-model.xlsx
+++ b/models/builds/2026-08-08-Kaetsu-eur-receivable-model.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="123">
   <si>
     <t xml:space="preserve">FX Hedging Model — EUR 4,500,000 Receivable</t>
   </si>
@@ -221,31 +221,28 @@
     <t xml:space="preserve">USD per EUR</t>
   </si>
   <si>
-    <t xml:space="preserve">Indicative — live spot from a market data provider (e.g. OANDA, Bloomberg) at Stage 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicative — quoted 1-year forward rate at Stage 4</t>
+    <t xml:space="preserve">LIVE — Bloomberg EURUSD quote, 1.1561, as of 2:23 PM EDT 08/07/2026 (bloomberg.com/quote/EURUSD:CUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIVE (CIP-implied) — no live 1-year forward quote found; computed via F0 = S0_in*(1+R_USD*T/360)/(1+R_FC*T/360)</t>
   </si>
   <si>
     <t xml:space="preserve">Annual % (ACT/360)</t>
   </si>
   <si>
-    <t xml:space="preserve">Indicative — Federal Reserve H.15 release (1-year rate) at Stage 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicative — ECB deposit facility rate at Stage 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicative — at-the-money to spot; refined against live option quotes at Stage 4</t>
+    <t xml:space="preserve">LIVE — 1-Year Treasury yield, 4.06%, Treasury.gov Daily Par Yield Curve Rates as of 2026-08-06 (via slickcharts.com/treasury)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIVE — ECB Deposit Facility Rate, 2.25%, ECB Data Portal, as of 02 Aug 2026, last updated 2026-08-02 01:38 CEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIVE — set at-the-money to live spot (S0_in = 1.1561), per scenario convention</t>
   </si>
   <si>
     <t xml:space="preserve">USD per unit FC</t>
   </si>
   <si>
-    <t xml:space="preserve">Indicative — quoted put premium at Stage 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicative — quoted call premium at Stage 4</t>
+    <t xml:space="preserve">ASSUMPTION — kept at scenario-given value; retail-accessible EUR option premium quotes are unreliable for this exercise</t>
   </si>
   <si>
     <t xml:space="preserve">Days</t>
@@ -605,16 +602,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -622,11 +623,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -634,27 +635,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -662,39 +663,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -702,11 +703,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -714,7 +715,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -864,22 +865,26 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -935,37 +940,37 @@
                 <c:formatCode>\$#,##0</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4965300</c:v>
+                  <c:v>5295600</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1002,22 +1007,26 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1073,37 +1082,37 @@
                 <c:formatCode>\$#,##0</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4965101.59837335</c:v>
+                  <c:v>5295792.80048885</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1140,22 +1149,26 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1211,37 +1224,37 @@
                 <c:formatCode>\$#,##0</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>4747500</c:v>
+                  <c:v>5089950</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4747500</c:v>
+                  <c:v>5089950</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4747500</c:v>
+                  <c:v>5089950</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4747500</c:v>
+                  <c:v>5089950</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4747500</c:v>
+                  <c:v>5089950</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4747500</c:v>
+                  <c:v>5089950</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4796100</c:v>
+                  <c:v>5141974.5</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4844700</c:v>
+                  <c:v>5193999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4893300</c:v>
+                  <c:v>5246023.5</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4941900</c:v>
+                  <c:v>5298048</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4990500</c:v>
+                  <c:v>5350072.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1256,11 +1269,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="56092219"/>
-        <c:axId val="59037259"/>
+        <c:axId val="79423914"/>
+        <c:axId val="43796832"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="56092219"/>
+        <c:axId val="79423914"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1300,7 +1313,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1326,7 +1339,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59037259"/>
+        <c:crossAx val="43796832"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1334,7 +1347,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59037259"/>
+        <c:axId val="43796832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1384,7 +1397,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="\$#,##0" sourceLinked="1"/>
+        <c:numFmt formatCode="\$#,##0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1410,7 +1423,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56092219"/>
+        <c:crossAx val="79423914"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1473,9 +1486,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>364680</xdr:colOff>
+      <xdr:colOff>364320</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>172080</xdr:rowOff>
+      <xdr:rowOff>171720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1483,8 +1496,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5968440" y="571680"/>
-        <a:ext cx="6479640" cy="3239640"/>
+        <a:off x="5968440" y="569160"/>
+        <a:ext cx="6479280" cy="3231720"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1680,114 +1693,114 @@
   <dimension ref="B2:C17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="80"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="2" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="2" t="s">
+    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="2" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="2" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="2" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="2" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1810,138 +1823,138 @@
   <dimension ref="B2:C21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="65"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="6" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="7"/>
-      <c r="C5" s="8" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="8"/>
+      <c r="C5" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="9"/>
-      <c r="C6" s="8" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="10"/>
+      <c r="C6" s="9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="10"/>
-      <c r="C7" s="8" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="11"/>
+      <c r="C7" s="9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="11"/>
-      <c r="C8" s="8" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="12"/>
+      <c r="C8" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="2" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="4" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="4" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="4" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="4" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1964,178 +1977,178 @@
   <dimension ref="B2:E17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="6" t="s">
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="13" t="n">
         <v>4500000</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="2" t="s">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="14" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="15" t="n">
+        <v>1.1561</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="14" t="n">
-        <v>1.1034</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="15" t="n">
+        <v>1.1768</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="2" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="15" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="16" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="2" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="15" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="16" t="n">
+        <v>0.0225</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="2" t="s">
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="15" t="n">
+        <v>1.1561</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="14" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="2" t="s">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="15" t="n">
+        <v>1.1561</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>0.025</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <v>0.022</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>365</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="16" t="n">
-        <v>365</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="13" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="18" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2159,31 +2172,31 @@
   <dimension ref="B2:C6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="19" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="20" t="n">
         <f aca="false">FC_AMT*F0_in</f>
-        <v>4965300</v>
+        <v>5295600</v>
       </c>
     </row>
   </sheetData>
@@ -2205,101 +2218,101 @@
   <dimension ref="B2:D14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="7" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="21" t="n">
+        <f aca="false">FC_AMT/(1+R_FC*T_DAYS/360)</f>
+        <v>4399633.36388634</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="20" t="n">
-        <f aca="false">FC_AMT/(1+R_FC*T_DAYS/360)</f>
-        <v>4362872.49370481</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="20" t="n">
+        <f aca="false">Borrow_FC*S0_in</f>
+        <v>5086416.131989</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D6" s="19" t="n">
-        <f aca="false">Borrow_FC*S0_in</f>
-        <v>4711902.29320119</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="20" t="n">
+        <f aca="false">USD_Now*(1+R_USD*T_DAYS/360)</f>
+        <v>5295792.80048885</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="19" t="n">
-        <f aca="false">USD_Now*(1+R_USD*T_DAYS/360)</f>
-        <v>4965101.59837335</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="18" t="s">
+      <c r="D9" s="22" t="n">
+        <f aca="false">Proceeds_MM</f>
+        <v>5295792.80048885</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D9" s="21" t="n">
-        <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="5" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="2" t="s">
+      <c r="D12" s="23" t="n">
+        <f aca="false">S0_in*(1+R_USD*T_DAYS/360)/(1+R_FC*T_DAYS/360)</f>
+        <v>1.17684284455308</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D12" s="22" t="n">
-        <f aca="false">S0_in*(1+R_USD*T_DAYS/360)/(1+R_FC*T_DAYS/360)</f>
-        <v>1.10335591074963</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="23" t="n">
+        <f aca="false">F0_in</f>
+        <v>1.1768</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="D13" s="22" t="n">
-        <f aca="false">F0_in</f>
-        <v>1.1034</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="D14" s="11" t="str">
+      <c r="D14" s="12" t="str">
         <f aca="false">IF(ABS(F_implied-F0_in)&lt;=0.001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
@@ -2323,187 +2336,187 @@
   <dimension ref="B2:D17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="7" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D4" s="6" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="23" t="n">
+        <f aca="false">S0_in*0.95</f>
+        <v>1.098295</v>
+      </c>
+      <c r="C5" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B5,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5089950</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B5,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>4843327.5</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="23" t="n">
+        <f aca="false">S0_in*0.96</f>
+        <v>1.109856</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B6,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5089950</v>
+      </c>
+      <c r="D6" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B6,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>4895352</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="23" t="n">
+        <f aca="false">S0_in*0.97</f>
+        <v>1.121417</v>
+      </c>
+      <c r="C7" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B7,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5089950</v>
+      </c>
+      <c r="D7" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B7,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>4947376.5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="23" t="n">
+        <f aca="false">S0_in*0.98</f>
+        <v>1.132978</v>
+      </c>
+      <c r="C8" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B8,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5089950</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B8,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>4999401</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="23" t="n">
+        <f aca="false">S0_in*0.99</f>
+        <v>1.144539</v>
+      </c>
+      <c r="C9" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B9,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5089950</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B9,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>5051425.5</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="23" t="n">
+        <f aca="false">S0_in*1</f>
+        <v>1.1561</v>
+      </c>
+      <c r="C10" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B10,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5089950</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B10,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>5103450</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="23" t="n">
+        <f aca="false">S0_in*1.01</f>
+        <v>1.167661</v>
+      </c>
+      <c r="C11" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B11,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5141974.5</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B11,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>5103450</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="23" t="n">
+        <f aca="false">S0_in*1.02</f>
+        <v>1.179222</v>
+      </c>
+      <c r="C12" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B12,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5193999</v>
+      </c>
+      <c r="D12" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B12,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>5103450</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="23" t="n">
+        <f aca="false">S0_in*1.03</f>
+        <v>1.190783</v>
+      </c>
+      <c r="C13" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B13,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5246023.5</v>
+      </c>
+      <c r="D13" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B13,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>5103450</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="23" t="n">
+        <f aca="false">S0_in*1.04</f>
+        <v>1.202344</v>
+      </c>
+      <c r="C14" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B14,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5298048</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B14,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>5103450</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="23" t="n">
+        <f aca="false">S0_in*1.05</f>
+        <v>1.213905</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <f aca="false">FC_AMT*MAX(B15,K_PUT)-FC_AMT*PREM_PUT</f>
+        <v>5350072.5</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <f aca="false">FC_AMT*MIN(B15,K_CALL)-FC_AMT*PREM_CALL</f>
+        <v>5103450</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="24" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="22" t="n">
-        <f aca="false">S0_in*0.95</f>
-        <v>1.026</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B5,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-      <c r="D5" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B5,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4518000</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="22" t="n">
-        <f aca="false">S0_in*0.96</f>
-        <v>1.0368</v>
-      </c>
-      <c r="C6" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B6,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-      <c r="D6" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B6,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4566600</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="22" t="n">
-        <f aca="false">S0_in*0.97</f>
-        <v>1.0476</v>
-      </c>
-      <c r="C7" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B7,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-      <c r="D7" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B7,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4615200</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="22" t="n">
-        <f aca="false">S0_in*0.98</f>
-        <v>1.0584</v>
-      </c>
-      <c r="C8" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B8,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-      <c r="D8" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B8,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4663800</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="22" t="n">
-        <f aca="false">S0_in*0.99</f>
-        <v>1.0692</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B9,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-      <c r="D9" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B9,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4712400</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="22" t="n">
-        <f aca="false">S0_in*1</f>
-        <v>1.08</v>
-      </c>
-      <c r="C10" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B10,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-      <c r="D10" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B10,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4761000</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="22" t="n">
-        <f aca="false">S0_in*1.01</f>
-        <v>1.0908</v>
-      </c>
-      <c r="C11" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B11,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4796100</v>
-      </c>
-      <c r="D11" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B11,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4761000</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="22" t="n">
-        <f aca="false">S0_in*1.02</f>
-        <v>1.1016</v>
-      </c>
-      <c r="C12" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B12,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4844700</v>
-      </c>
-      <c r="D12" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B12,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4761000</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="22" t="n">
-        <f aca="false">S0_in*1.03</f>
-        <v>1.1124</v>
-      </c>
-      <c r="C13" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B13,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4893300</v>
-      </c>
-      <c r="D13" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B13,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4761000</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="22" t="n">
-        <f aca="false">S0_in*1.04</f>
-        <v>1.1232</v>
-      </c>
-      <c r="C14" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B14,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4941900</v>
-      </c>
-      <c r="D14" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B14,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4761000</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="22" t="n">
-        <f aca="false">S0_in*1.05</f>
-        <v>1.134</v>
-      </c>
-      <c r="C15" s="19" t="n">
-        <f aca="false">FC_AMT*MAX(B15,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4990500</v>
-      </c>
-      <c r="D15" s="19" t="n">
-        <f aca="false">FC_AMT*MIN(B15,K_CALL)-FC_AMT*PREM_CALL</f>
-        <v>4761000</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2527,263 +2540,263 @@
   <dimension ref="B2:F15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="7" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="24" t="n">
+      <c r="D4" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="25" t="n">
         <v>-0.05</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="23" t="n">
         <f aca="false">S0_in*(1+B5)</f>
-        <v>1.026</v>
-      </c>
-      <c r="D5" s="19" t="n">
+        <v>1.098295</v>
+      </c>
+      <c r="D5" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E5" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E5" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F5" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F5" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C5,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="24" t="n">
+        <v>5089950</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="25" t="n">
         <v>-0.04</v>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="23" t="n">
         <f aca="false">S0_in*(1+B6)</f>
-        <v>1.0368</v>
-      </c>
-      <c r="D6" s="19" t="n">
+        <v>1.109856</v>
+      </c>
+      <c r="D6" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E6" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E6" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F6" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F6" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C6,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="24" t="n">
+        <v>5089950</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="25" t="n">
         <v>-0.03</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <f aca="false">S0_in*(1+B7)</f>
-        <v>1.0476</v>
-      </c>
-      <c r="D7" s="19" t="n">
+        <v>1.121417</v>
+      </c>
+      <c r="D7" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E7" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E7" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F7" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F7" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C7,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="24" t="n">
+        <v>5089950</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="25" t="n">
         <v>-0.02</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <f aca="false">S0_in*(1+B8)</f>
-        <v>1.0584</v>
-      </c>
-      <c r="D8" s="19" t="n">
+        <v>1.132978</v>
+      </c>
+      <c r="D8" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E8" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E8" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F8" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F8" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C8,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="24" t="n">
+        <v>5089950</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="25" t="n">
         <v>-0.01</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <f aca="false">S0_in*(1+B9)</f>
-        <v>1.0692</v>
-      </c>
-      <c r="D9" s="19" t="n">
+        <v>1.144539</v>
+      </c>
+      <c r="D9" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E9" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E9" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F9" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F9" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C9,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="24" t="n">
+        <v>5089950</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <f aca="false">S0_in*(1+B10)</f>
-        <v>1.08</v>
-      </c>
-      <c r="D10" s="19" t="n">
+        <v>1.1561</v>
+      </c>
+      <c r="D10" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E10" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F10" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F10" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C10,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4747500</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="24" t="n">
+        <v>5089950</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="25" t="n">
         <v>0.01</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="23" t="n">
         <f aca="false">S0_in*(1+B11)</f>
-        <v>1.0908</v>
-      </c>
-      <c r="D11" s="19" t="n">
+        <v>1.167661</v>
+      </c>
+      <c r="D11" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E11" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F11" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F11" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C11,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4796100</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="24" t="n">
+        <v>5141974.5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="25" t="n">
         <v>0.02</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <f aca="false">S0_in*(1+B12)</f>
-        <v>1.1016</v>
-      </c>
-      <c r="D12" s="19" t="n">
+        <v>1.179222</v>
+      </c>
+      <c r="D12" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E12" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F12" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F12" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C12,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4844700</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="24" t="n">
+        <v>5193999</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="25" t="n">
         <v>0.03</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <f aca="false">S0_in*(1+B13)</f>
-        <v>1.1124</v>
-      </c>
-      <c r="D13" s="19" t="n">
+        <v>1.190783</v>
+      </c>
+      <c r="D13" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E13" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E13" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F13" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F13" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C13,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4893300</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="24" t="n">
+        <v>5246023.5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="25" t="n">
         <v>0.04</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="23" t="n">
         <f aca="false">S0_in*(1+B14)</f>
-        <v>1.1232</v>
-      </c>
-      <c r="D14" s="19" t="n">
+        <v>1.202344</v>
+      </c>
+      <c r="D14" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E14" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E14" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F14" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F14" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C14,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4941900</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="24" t="n">
+        <v>5298048</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="25" t="n">
         <v>0.05</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="23" t="n">
         <f aca="false">S0_in*(1+B15)</f>
-        <v>1.134</v>
-      </c>
-      <c r="D15" s="19" t="n">
+        <v>1.213905</v>
+      </c>
+      <c r="D15" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>4965300</v>
-      </c>
-      <c r="E15" s="19" t="n">
+        <v>5295600</v>
+      </c>
+      <c r="E15" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>4965101.59837335</v>
-      </c>
-      <c r="F15" s="19" t="n">
+        <v>5295792.80048885</v>
+      </c>
+      <c r="F15" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C15,K_PUT)-FC_AMT*PREM_PUT</f>
-        <v>4990500</v>
+        <v>5350072.5</v>
       </c>
     </row>
   </sheetData>
@@ -2806,130 +2819,130 @@
   <dimension ref="B2:D16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="26" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="25" t="s">
+      <c r="C4" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="26" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="26" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="25" t="s">
+      <c r="C5" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="C5" s="26" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="26" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="25" t="s">
+      <c r="C6" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="26" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="26" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="25" t="s">
+      <c r="C7" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="C7" s="26" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="6" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="D10" s="2" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="5" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D11" s="27" t="str">
+      <c r="D11" s="28" t="str">
         <f aca="false">'Money Market'!D14</f>
         <v>PASS</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="27" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="5" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="D13" s="27" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="5" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="D14" s="27" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="5" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="28" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="27" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="5" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="28" t="s">
         <v>122</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct R_FC to tenor-matched rate per Treasury review
</commit_message>
<xml_diff>
--- a/models/builds/2026-08-08-Kaetsu-eur-receivable-model.xlsx
+++ b/models/builds/2026-08-08-Kaetsu-eur-receivable-model.xlsx
@@ -224,7 +224,7 @@
     <t xml:space="preserve">LIVE — Bloomberg EURUSD quote, 1.1561, as of 2:23 PM EDT 08/07/2026 (bloomberg.com/quote/EURUSD:CUR)</t>
   </si>
   <si>
-    <t xml:space="preserve">LIVE (CIP-implied) — no live 1-year forward quote found; computed via F0 = S0_in*(1+R_USD*T/360)/(1+R_FC*T/360)</t>
+    <t xml:space="preserve">LIVE (CIP-implied, recomputed) — no live 1-year forward quote found; F0 = S0_in*(1+R_USD*T/360)/(1+R_FC*T/360) using the corrected tenor-matched R_FC</t>
   </si>
   <si>
     <t xml:space="preserve">Annual % (ACT/360)</t>
@@ -233,7 +233,7 @@
     <t xml:space="preserve">LIVE — 1-Year Treasury yield, 4.06%, Treasury.gov Daily Par Yield Curve Rates as of 2026-08-06 (via slickcharts.com/treasury)</t>
   </si>
   <si>
-    <t xml:space="preserve">LIVE — ECB Deposit Facility Rate, 2.25%, ECB Data Portal, as of 02 Aug 2026, last updated 2026-08-02 01:38 CEST</t>
+    <t xml:space="preserve">LIVE (CORRECTED) — Eurostat/ECB euro area 1-year yield curve, 2.01%, Dec 2025 reading (most recent published; tenor-matched to T_DAYS=365, replacing the overnight ECB deposit facility rate used in the initial Stage 4 pull per Treasury review)</t>
   </si>
   <si>
     <t xml:space="preserve">LIVE — set at-the-money to live spot (S0_in = 1.1561), per scenario convention</t>
@@ -940,37 +940,37 @@
                 <c:formatCode>\$#,##0</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5295600</c:v>
+                  <c:v>5308200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1082,37 +1082,37 @@
                 <c:formatCode>\$#,##0</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5295792.80048885</c:v>
+                  <c:v>5308421.85992952</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1269,11 +1269,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="79423914"/>
-        <c:axId val="43796832"/>
+        <c:axId val="56867198"/>
+        <c:axId val="13983496"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="79423914"/>
+        <c:axId val="56867198"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1339,7 +1339,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43796832"/>
+        <c:crossAx val="13983496"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1347,7 +1347,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="43796832"/>
+        <c:axId val="13983496"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1423,7 +1423,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79423914"/>
+        <c:crossAx val="56867198"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1486,9 +1486,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>364320</xdr:colOff>
+      <xdr:colOff>363960</xdr:colOff>
       <xdr:row>18</xdr:row>
-      <xdr:rowOff>171720</xdr:rowOff>
+      <xdr:rowOff>171360</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1497,7 +1497,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="5968440" y="569160"/>
-        <a:ext cx="6479280" cy="3231720"/>
+        <a:ext cx="6478920" cy="3231360"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2035,7 +2035,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>1.1768</v>
+        <v>1.1796</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>57</v>
@@ -2063,7 +2063,7 @@
         <v>18</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>0.0225</v>
+        <v>0.0201</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>60</v>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C6" s="20" t="n">
         <f aca="false">FC_AMT*F0_in</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
     </row>
   </sheetData>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="D5" s="21" t="n">
         <f aca="false">FC_AMT/(1+R_FC*T_DAYS/360)</f>
-        <v>4399633.36388634</v>
+        <v>4410125.32106121</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="D6" s="20" t="n">
         <f aca="false">Borrow_FC*S0_in</f>
-        <v>5086416.131989</v>
+        <v>5098545.88367886</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="D7" s="20" t="n">
         <f aca="false">USD_Now*(1+R_USD*T_DAYS/360)</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D9" s="22" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="D12" s="23" t="n">
         <f aca="false">S0_in*(1+R_USD*T_DAYS/360)/(1+R_FC*T_DAYS/360)</f>
-        <v>1.17684284455308</v>
+        <v>1.17964930220656</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="D13" s="23" t="n">
         <f aca="false">F0_in</f>
-        <v>1.1768</v>
+        <v>1.1796</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2578,11 +2578,11 @@
       </c>
       <c r="D5" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E5" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F5" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C5,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2599,11 +2599,11 @@
       </c>
       <c r="D6" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F6" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C6,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2620,11 +2620,11 @@
       </c>
       <c r="D7" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F7" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C7,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2641,11 +2641,11 @@
       </c>
       <c r="D8" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E8" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F8" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C8,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2662,11 +2662,11 @@
       </c>
       <c r="D9" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E9" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F9" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C9,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2683,11 +2683,11 @@
       </c>
       <c r="D10" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E10" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F10" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C10,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2704,11 +2704,11 @@
       </c>
       <c r="D11" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E11" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F11" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C11,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2725,11 +2725,11 @@
       </c>
       <c r="D12" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E12" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F12" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C12,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2746,11 +2746,11 @@
       </c>
       <c r="D13" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E13" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F13" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C13,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2767,11 +2767,11 @@
       </c>
       <c r="D14" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E14" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F14" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C14,K_PUT)-FC_AMT*PREM_PUT</f>
@@ -2788,11 +2788,11 @@
       </c>
       <c r="D15" s="20" t="n">
         <f aca="false">Proceeds_Forward</f>
-        <v>5295600</v>
+        <v>5308200</v>
       </c>
       <c r="E15" s="20" t="n">
         <f aca="false">Proceeds_MM</f>
-        <v>5295792.80048885</v>
+        <v>5308421.85992952</v>
       </c>
       <c r="F15" s="20" t="n">
         <f aca="false">FC_AMT*MAX(C15,K_PUT)-FC_AMT*PREM_PUT</f>

</xml_diff>